<commit_message>
refactor and code logic changes
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/CourseData.xlsx
+++ b/src/test/resources/testdata/CourseData.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
-    <t>Extracted: 18-May-2026 14:30:34</t>
+    <t>Extracted: 18-May-2026 22:58:01</t>
   </si>
   <si>
     <t>S.No</t>
@@ -38,16 +38,16 @@
     <t>4.7</t>
   </si>
   <si>
+    <t>Introduction to Web Development with HTML, CSS, JavaScript</t>
+  </si>
+  <si>
+    <t>1 - 3 Months</t>
+  </si>
+  <si>
+    <t>4.6</t>
+  </si>
+  <si>
     <t>Front-End Web Development for Beginners</t>
-  </si>
-  <si>
-    <t>1 - 3 Months</t>
-  </si>
-  <si>
-    <t>4.6</t>
-  </si>
-  <si>
-    <t>Introduction to Web Development with HTML, CSS, JavaScript</t>
   </si>
   <si>
     <t>Introduction to HTML, CSS, &amp; JavaScript</t>

</xml_diff>

<commit_message>
refactored code and optimized the logic
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/CourseData.xlsx
+++ b/src/test/resources/testdata/CourseData.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
-    <t>Extracted: 18-May-2026 22:58:01</t>
+    <t>Extracted: 19-May-2026 13:41:01</t>
   </si>
   <si>
     <t>S.No</t>
@@ -29,7 +29,7 @@
     <t>Rating</t>
   </si>
   <si>
-    <t>Web Development for Beginners</t>
+    <t>Status: Free Trial</t>
   </si>
   <si>
     <t>3 - 6 Months</t>
@@ -38,7 +38,7 @@
     <t>4.7</t>
   </si>
   <si>
-    <t>Introduction to Web Development with HTML, CSS, JavaScript</t>
+    <t>Status: Preview</t>
   </si>
   <si>
     <t>1 - 3 Months</t>
@@ -47,19 +47,10 @@
     <t>4.6</t>
   </si>
   <si>
-    <t>Front-End Web Development for Beginners</t>
+    <t>Status: New</t>
   </si>
   <si>
-    <t>Introduction to HTML, CSS, &amp; JavaScript</t>
-  </si>
-  <si>
-    <t>1 - 4 Weeks</t>
-  </si>
-  <si>
-    <t>4.4</t>
-  </si>
-  <si>
-    <t>Introduction to Web Development</t>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -104,11 +95,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="27.765625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="50.5078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="14.390625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="13.04296875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="6.02734375" customWidth="true" bestFit="true"/>
   </cols>
@@ -168,38 +159,10 @@
         <v>11</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n" s="0">
-        <v>4.0</v>
-      </c>
-      <c r="B6" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n" s="0">
-        <v>5.0</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final Version of the Project
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/CourseData.xlsx
+++ b/src/test/resources/testdata/CourseData.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
-  <si>
-    <t>Extracted: 19-May-2026 13:41:01</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+  <si>
+    <t>Extracted: 22-May-2026 17:40:31</t>
   </si>
   <si>
     <t>S.No</t>
@@ -29,7 +29,7 @@
     <t>Rating</t>
   </si>
   <si>
-    <t>Status: Free Trial</t>
+    <t>Web Development for Beginners</t>
   </si>
   <si>
     <t>3 - 6 Months</t>
@@ -38,7 +38,7 @@
     <t>4.7</t>
   </si>
   <si>
-    <t>Status: Preview</t>
+    <t>Introduction to Web Development with HTML, CSS, JavaScript</t>
   </si>
   <si>
     <t>1 - 3 Months</t>
@@ -47,10 +47,22 @@
     <t>4.6</t>
   </si>
   <si>
-    <t>Status: New</t>
+    <t>Front-End Web Development for Beginners</t>
+  </si>
+  <si>
+    <t>Introduction to Web Development and HTML Basics</t>
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Introduction to HTML, CSS, &amp; JavaScript</t>
+  </si>
+  <si>
+    <t>1 - 4 Weeks</t>
+  </si>
+  <si>
+    <t>4.4</t>
   </si>
 </sst>
 </file>
@@ -95,11 +107,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="27.765625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="14.390625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="50.5078125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="13.04296875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="6.02734375" customWidth="true" bestFit="true"/>
   </cols>
@@ -159,10 +171,38 @@
         <v>11</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
         <v>12</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>